<commit_message>
feat: complete Face Recognition Attendance System with multi-angle capture and registration portal
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,17 +436,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>roll_no</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>time</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>
@@ -456,17 +471,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Parmjeet</t>
+          <t>STU-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>PARMJEET</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>16:42:23</t>
+          <t>B.Tech (CSE)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>02:05:28</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Present</t>
         </is>
       </c>
     </row>
@@ -476,77 +506,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Parmjeet</t>
+          <t>STU-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>MUKUL THAKUR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16:43:21</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Parmjeet</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2025-12-27</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>16:43:26</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Parmjeet</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2025-12-27</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>16:48:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Parmjeet</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2025-12-27</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>16:48:15</t>
+          <t>B.Tech (CSE)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>02:16:30</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Present</t>
         </is>
       </c>
     </row>

</xml_diff>